<commit_message>
Script de ejercicio 1 modificado para aceptar argumentos para ejecutar estudiantes o inventario.
</commit_message>
<xml_diff>
--- a/practicaPython/tallerFinal/Ejercicio1/repo/estudiantes.xlsx
+++ b/practicaPython/tallerFinal/Ejercicio1/repo/estudiantes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,6 +461,21 @@
       </c>
       <c r="C3" t="n">
         <v>18.53</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Adrian</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mercadotecnia</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>17.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>